<commit_message>
Add links to judge prompts to random eval xlsx
</commit_message>
<xml_diff>
--- a/src/scripts/random_eval_1.xlsx
+++ b/src/scripts/random_eval_1.xlsx
@@ -28,14 +28,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-    </font>
-    <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="10"/>
       <sz val="12"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -57,15 +57,18 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -463,64 +466,25 @@
             <t xml:space="preserve">0. </t>
           </r>
           <r>
-            <t>Review the JudgeSystem and JudgeUser prompts to understand the criteria used during realism evaluation.</t>
+            <t>Review the following prompts to understand the criteria used during realism evaluation.</t>
           </r>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t xml:space="preserve">1. </t>
-          </r>
-          <r>
-            <t>Open and review the instance from the hyperlink in the first column.</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <r>
+            <t>System Judge: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=system-judge-prompt</t>
           </r>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t xml:space="preserve">2. </t>
-          </r>
-          <r>
-            <t xml:space="preserve">In your corresponding reviewer column, write </t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t>'R'</t>
-          </r>
-          <r>
-            <t xml:space="preserve"> (realistic), </t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t>'U'</t>
-          </r>
-          <r>
-            <t xml:space="preserve"> (unrealistic), or </t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t>'D'</t>
-          </r>
-          <r>
-            <t xml:space="preserve"> (doubtful).</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <r>
+            <t>User Judge: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=user-judge-prompt</t>
           </r>
         </is>
       </c>
@@ -532,16 +496,10 @@
             <rPr>
               <b val="1"/>
             </rPr>
-            <t xml:space="preserve">3. </t>
-          </r>
-          <r>
-            <t xml:space="preserve">Add a short explanation only for U or D, for example: </t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t>'U: It is implausible to make an omelet without eggs.'</t>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <t>Open and review the instance from the hyperlink in the first column.</t>
           </r>
         </is>
       </c>
@@ -550,6 +508,69 @@
       <c r="A6" s="1" t="inlineStr">
         <is>
           <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">2. </t>
+          </r>
+          <r>
+            <t xml:space="preserve">In your corresponding reviewer column, write </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>'R'</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (realistic), </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>'U'</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (unrealistic), or </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>'D'</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (doubtful).</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">3. </t>
+          </r>
+          <r>
+            <t xml:space="preserve">Add a short explanation only for U or D, for example: </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>'U: It is implausible to make an omelet without eggs.'</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <r>
             <t xml:space="preserve">Another valid example: </t>
           </r>
           <r>
@@ -561,40 +582,8 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Instance Id</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Lola</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Dominik</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Manuel</t>
-        </is>
-      </c>
-    </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / myexpenses / gen15</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
@@ -602,17 +591,29 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / myexpenses / gen11</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+          <t>Instance Id</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Lola</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Dominik</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Manuel</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / bank / gen2 / baseline</t>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / myexpenses / gen15</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -620,9 +621,9 @@
       <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / pickupnet / gen11</t>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / myexpenses / gen11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -630,9 +631,9 @@
       <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / pickupnet / gen28</t>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / bank / gen2 / baseline</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -640,9 +641,9 @@
       <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / myexpenses / gen5 / baseline</t>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / pickupnet / gen11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -650,9 +651,9 @@
       <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / vehiclerental / gen6 / complex</t>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / pickupnet / gen28</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -660,9 +661,9 @@
       <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / restaurant / gen26</t>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / myexpenses / gen5 / baseline</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -670,9 +671,9 @@
       <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / videoclub / gen6</t>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / vehiclerental / gen6 / complex</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -680,9 +681,9 @@
       <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / restaurant / gen4 / complex</t>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / restaurant / gen26</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -690,9 +691,9 @@
       <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / bank / gen13</t>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / videoclub / gen6</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -700,9 +701,9 @@
       <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / myexpenses / gen5 / invalid</t>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / restaurant / gen4 / complex</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -710,9 +711,9 @@
       <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / statemachine / gen4</t>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / bank / gen13</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -720,9 +721,9 @@
       <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / videoclub / gen5 / boundary</t>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / myexpenses / gen5 / invalid</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -730,9 +731,9 @@
       <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / football / gen1 / boundary</t>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / statemachine / gen4</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -740,9 +741,9 @@
       <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / pickupnet / gen4 / boundary</t>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / videoclub / gen5 / boundary</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -750,9 +751,9 @@
       <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / restaurant / gen20</t>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / football / gen1 / boundary</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -760,9 +761,9 @@
       <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / videoclub / gen16</t>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / pickupnet / gen4 / boundary</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -770,9 +771,9 @@
       <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / addressbook / gen10</t>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / restaurant / gen20</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -780,9 +781,9 @@
       <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / hotelmanagement / gen1 / edge</t>
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / videoclub / gen16</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -790,9 +791,9 @@
       <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / restaurant / gen6 / boundary</t>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / addressbook / gen10</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -800,9 +801,9 @@
       <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / vehiclerental / gen27</t>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / hotelmanagement / gen1 / edge</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -810,9 +811,9 @@
       <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / addressbook / gen26</t>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / restaurant / gen6 / boundary</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -820,27 +821,49 @@
       <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / statemachine / gen3</t>
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / vehiclerental / gen27</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
     </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / addressbook / gen26</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / statemachine / gen3</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A8:D8"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A7:D7"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId5"/>
@@ -863,6 +886,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -874,7 +899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -905,64 +930,25 @@
             <t xml:space="preserve">0. </t>
           </r>
           <r>
-            <t>Review the JudgeSystem and JudgeUser prompts to understand the criteria used during realism evaluation.</t>
+            <t>Review the following prompts to understand the criteria used during realism evaluation.</t>
           </r>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t xml:space="preserve">1. </t>
-          </r>
-          <r>
-            <t>Open and review the instance from the hyperlink in the first column.</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <r>
+            <t>System Judge: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=system-judge-prompt</t>
           </r>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t xml:space="preserve">2. </t>
-          </r>
-          <r>
-            <t xml:space="preserve">In your corresponding reviewer column, write </t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t>'R'</t>
-          </r>
-          <r>
-            <t xml:space="preserve"> (realistic), </t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t>'U'</t>
-          </r>
-          <r>
-            <t xml:space="preserve"> (unrealistic), or </t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t>'D'</t>
-          </r>
-          <r>
-            <t xml:space="preserve"> (doubtful).</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <r>
+            <t>User Judge: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=user-judge-prompt</t>
           </r>
         </is>
       </c>
@@ -974,16 +960,10 @@
             <rPr>
               <b val="1"/>
             </rPr>
-            <t xml:space="preserve">3. </t>
-          </r>
-          <r>
-            <t xml:space="preserve">Add a short explanation only for U or D, for example: </t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t>'U: It is implausible to make an omelet without eggs.'</t>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <t>Open and review the instance from the hyperlink in the first column.</t>
           </r>
         </is>
       </c>
@@ -992,6 +972,69 @@
       <c r="A6" s="1" t="inlineStr">
         <is>
           <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">2. </t>
+          </r>
+          <r>
+            <t xml:space="preserve">In your corresponding reviewer column, write </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>'R'</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (realistic), </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>'U'</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (unrealistic), or </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>'D'</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (doubtful).</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">3. </t>
+          </r>
+          <r>
+            <t xml:space="preserve">Add a short explanation only for U or D, for example: </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>'U: It is implausible to make an omelet without eggs.'</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <r>
             <t xml:space="preserve">Another valid example: </t>
           </r>
           <r>
@@ -1003,40 +1046,8 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Instance Id</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Lola</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Manuel</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Dominik</t>
-        </is>
-      </c>
-    </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / videoclub / gen2 / baseline</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
@@ -1044,17 +1055,29 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / videoclub / gen2 / complex</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+          <t>Instance Id</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Lola</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Manuel</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Dominik</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / bank / gen5 / boundary</t>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / videoclub / gen2 / baseline</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -1062,9 +1085,9 @@
       <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / statemachine / gen20</t>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / videoclub / gen2 / complex</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -1072,9 +1095,9 @@
       <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / myexpenses / gen4 / baseline</t>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / bank / gen5 / boundary</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -1082,9 +1105,9 @@
       <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / videoclub / gen2 / baseline</t>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / statemachine / gen20</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -1092,9 +1115,9 @@
       <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / addressbook / gen17</t>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / myexpenses / gen4 / baseline</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -1102,9 +1125,9 @@
       <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / addressbook / gen20</t>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / videoclub / gen2 / baseline</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -1112,9 +1135,9 @@
       <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / addressbook / gen30</t>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / addressbook / gen17</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -1122,9 +1145,9 @@
       <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / restaurant / gen10</t>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / addressbook / gen20</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -1132,9 +1155,9 @@
       <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / football / gen21</t>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / addressbook / gen30</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -1142,9 +1165,9 @@
       <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / pickupnet / gen11</t>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / restaurant / gen10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -1152,9 +1175,9 @@
       <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / addressbook / gen1 / boundary</t>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / football / gen21</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -1162,9 +1185,9 @@
       <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / football / gen4 / boundary</t>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / pickupnet / gen11</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -1172,9 +1195,9 @@
       <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / football / gen2 / complex</t>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / addressbook / gen1 / boundary</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -1182,9 +1205,9 @@
       <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / vehiclerental / gen5 / boundary</t>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / football / gen4 / boundary</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -1192,9 +1215,9 @@
       <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / pickupnet / gen2</t>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / football / gen2 / complex</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -1202,9 +1225,9 @@
       <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / hotelmanagement / gen3 / baseline</t>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / vehiclerental / gen5 / boundary</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -1212,9 +1235,9 @@
       <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / addressbook / gen11</t>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / pickupnet / gen2</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -1222,9 +1245,9 @@
       <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / hotelmanagement / gen5 / complex</t>
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / hotelmanagement / gen3 / baseline</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -1232,9 +1255,9 @@
       <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / restaurant / gen1</t>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / addressbook / gen11</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -1242,9 +1265,9 @@
       <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / statemachine / gen1 / boundary</t>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / hotelmanagement / gen5 / complex</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1252,9 +1275,9 @@
       <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / pickupnet / gen23</t>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / restaurant / gen1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1262,27 +1285,49 @@
       <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / hotelmanagement / gen13</t>
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / statemachine / gen1 / boundary</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
     </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / pickupnet / gen23</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / hotelmanagement / gen13</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A8:D8"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A7:D7"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId5"/>
@@ -1305,6 +1350,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1316,7 +1363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1347,64 +1394,25 @@
             <t xml:space="preserve">0. </t>
           </r>
           <r>
-            <t>Review the JudgeSystem and JudgeUser prompts to understand the criteria used during realism evaluation.</t>
+            <t>Review the following prompts to understand the criteria used during realism evaluation.</t>
           </r>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t xml:space="preserve">1. </t>
-          </r>
-          <r>
-            <t>Open and review the instance from the hyperlink in the first column.</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <r>
+            <t>System Judge: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=system-judge-prompt</t>
           </r>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t xml:space="preserve">2. </t>
-          </r>
-          <r>
-            <t xml:space="preserve">In your corresponding reviewer column, write </t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t>'R'</t>
-          </r>
-          <r>
-            <t xml:space="preserve"> (realistic), </t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t>'U'</t>
-          </r>
-          <r>
-            <t xml:space="preserve"> (unrealistic), or </t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t>'D'</t>
-          </r>
-          <r>
-            <t xml:space="preserve"> (doubtful).</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <r>
+            <t>User Judge: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=user-judge-prompt</t>
           </r>
         </is>
       </c>
@@ -1416,16 +1424,10 @@
             <rPr>
               <b val="1"/>
             </rPr>
-            <t xml:space="preserve">3. </t>
-          </r>
-          <r>
-            <t xml:space="preserve">Add a short explanation only for U or D, for example: </t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t>'U: It is implausible to make an omelet without eggs.'</t>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <t>Open and review the instance from the hyperlink in the first column.</t>
           </r>
         </is>
       </c>
@@ -1434,6 +1436,69 @@
       <c r="A6" s="1" t="inlineStr">
         <is>
           <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">2. </t>
+          </r>
+          <r>
+            <t xml:space="preserve">In your corresponding reviewer column, write </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>'R'</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (realistic), </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>'U'</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (unrealistic), or </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>'D'</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (doubtful).</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">3. </t>
+          </r>
+          <r>
+            <t xml:space="preserve">Add a short explanation only for U or D, for example: </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>'U: It is implausible to make an omelet without eggs.'</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <r>
             <t xml:space="preserve">Another valid example: </t>
           </r>
           <r>
@@ -1445,40 +1510,8 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Instance Id</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Dominik</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Manuel</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Lola</t>
-        </is>
-      </c>
-    </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / pickupnet / gen4 / invalid</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
@@ -1486,17 +1519,29 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / restaurant / gen6 / edge</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+          <t>Instance Id</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Dominik</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Manuel</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Lola</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / vehiclerental / gen19</t>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / pickupnet / gen4 / invalid</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -1504,9 +1549,9 @@
       <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / football / gen8</t>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / restaurant / gen6 / edge</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -1514,9 +1559,9 @@
       <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / statemachine / gen2 / boundary</t>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / vehiclerental / gen19</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -1524,9 +1569,9 @@
       <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / statemachine / gen15</t>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / football / gen8</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -1534,9 +1579,9 @@
       <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / football / gen3 / complex</t>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / statemachine / gen2 / boundary</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -1544,9 +1589,9 @@
       <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / statemachine / gen29</t>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / statemachine / gen15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -1554,9 +1599,9 @@
       <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / videoclub / gen2 / edge</t>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / football / gen3 / complex</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -1564,9 +1609,9 @@
       <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / vehiclerental / gen8</t>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / statemachine / gen29</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -1574,9 +1619,9 @@
       <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / bank / gen20</t>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / videoclub / gen2 / edge</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -1584,9 +1629,9 @@
       <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / vehiclerental / gen21</t>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / vehiclerental / gen8</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -1594,9 +1639,9 @@
       <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / myexpenses / gen4 / edge</t>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / bank / gen20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -1604,9 +1649,9 @@
       <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / restaurant / gen2 / baseline</t>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / vehiclerental / gen21</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -1614,9 +1659,9 @@
       <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / hotelmanagement / gen1 / baseline</t>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / myexpenses / gen4 / edge</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -1624,9 +1669,9 @@
       <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / restaurant / gen3 / baseline</t>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / restaurant / gen2 / baseline</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -1634,9 +1679,9 @@
       <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / statemachine / gen3 / edge</t>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / hotelmanagement / gen1 / baseline</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -1644,9 +1689,9 @@
       <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / restaurant / gen8</t>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / restaurant / gen3 / baseline</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -1654,9 +1699,9 @@
       <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / simple / bank / gen17</t>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / statemachine / gen3 / edge</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -1664,9 +1709,9 @@
       <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / statemachine / gen4 / edge</t>
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / restaurant / gen8</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -1674,9 +1719,9 @@
       <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>gpt_4o / cot / statemachine / gen4 / baseline</t>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / simple / bank / gen17</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -1684,9 +1729,9 @@
       <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / hotelmanagement / gen6 / baseline</t>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / statemachine / gen4 / edge</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1694,9 +1739,9 @@
       <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / cot / pickupnet / gen4 / complex</t>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>gpt_4o / cot / statemachine / gen4 / baseline</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1704,27 +1749,49 @@
       <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>gpt_5_2 / simple / restaurant / gen11</t>
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / hotelmanagement / gen6 / baseline</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
     </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / cot / pickupnet / gen4 / complex</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>gpt_5_2 / simple / restaurant / gen11</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A8:D8"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A7:D7"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId5"/>
@@ -1747,6 +1814,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add docs and default seed constant
</commit_message>
<xml_diff>
--- a/src/scripts/random_eval_1.xlsx
+++ b/src/scripts/random_eval_1.xlsx
@@ -499,7 +499,7 @@
             <t xml:space="preserve">1. </t>
           </r>
           <r>
-            <t>Open and review the instance from the hyperlink in the first column.</t>
+            <t>Understand the model (diagram/code) and review the instance (diagram/code) from the hyperlink in the first column.</t>
           </r>
         </is>
       </c>
@@ -514,7 +514,7 @@
             <t xml:space="preserve">2. </t>
           </r>
           <r>
-            <t xml:space="preserve">In your corresponding reviewer column, write </t>
+            <t xml:space="preserve">In your corresponding reviewer excel, page and column, write </t>
           </r>
           <r>
             <rPr>
@@ -963,7 +963,7 @@
             <t xml:space="preserve">1. </t>
           </r>
           <r>
-            <t>Open and review the instance from the hyperlink in the first column.</t>
+            <t>Understand the model (diagram/code) and review the instance (diagram/code) from the hyperlink in the first column.</t>
           </r>
         </is>
       </c>
@@ -978,7 +978,7 @@
             <t xml:space="preserve">2. </t>
           </r>
           <r>
-            <t xml:space="preserve">In your corresponding reviewer column, write </t>
+            <t xml:space="preserve">In your corresponding reviewer excel, page and column, write </t>
           </r>
           <r>
             <rPr>
@@ -1427,7 +1427,7 @@
             <t xml:space="preserve">1. </t>
           </r>
           <r>
-            <t>Open and review the instance from the hyperlink in the first column.</t>
+            <t>Understand the model (diagram/code) and review the instance (diagram/code) from the hyperlink in the first column.</t>
           </r>
         </is>
       </c>
@@ -1442,7 +1442,7 @@
             <t xml:space="preserve">2. </t>
           </r>
           <r>
-            <t xml:space="preserve">In your corresponding reviewer column, write </t>
+            <t xml:space="preserve">In your corresponding reviewer excel, page and column, write </t>
           </r>
           <r>
             <rPr>

</xml_diff>

<commit_message>
Update random_eval scripts with the new judge.json. Move GPT_4o_old to Gemini 3 Pro judge model
</commit_message>
<xml_diff>
--- a/src/scripts/random_eval_1.xlsx
+++ b/src/scripts/random_eval_1.xlsx
@@ -466,7 +466,7 @@
             <t xml:space="preserve">0. </t>
           </r>
           <r>
-            <t>Review the following prompts to understand the criteria used during realism evaluation.</t>
+            <t>Review the judge prompts to understand the criteria used during realism evaluation.</t>
           </r>
         </is>
       </c>
@@ -475,7 +475,7 @@
       <c r="A3" s="2" t="inlineStr">
         <is>
           <r>
-            <t>System Judge: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=system-judge-prompt</t>
+            <t>Judge System Prompt: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=system-judge-prompt</t>
           </r>
         </is>
       </c>
@@ -484,7 +484,7 @@
       <c r="A4" s="2" t="inlineStr">
         <is>
           <r>
-            <t>User Judge: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=user-judge-prompt</t>
+            <t>Judge User Prompt: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=user-judge-prompt</t>
           </r>
         </is>
       </c>
@@ -613,7 +613,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / myexpenses / gen15</t>
+          <t>gpt_5_2 / simple / myexpenses / gen6</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -623,7 +623,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / myexpenses / gen11</t>
+          <t>gpt_5_2 / simple / bank / gen20</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -633,7 +633,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / bank / gen2 / baseline</t>
+          <t>gpt_5_2 / cot / bank / gen4 / complex</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -643,7 +643,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / pickupnet / gen11</t>
+          <t>gpt_5_2 / simple / pickupnet / gen13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -653,7 +653,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / pickupnet / gen28</t>
+          <t>gpt_4o / simple / pickupnet / gen29</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -663,7 +663,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / myexpenses / gen5 / baseline</t>
+          <t>gpt_5_2 / cot / myexpenses / gen5 / edge</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -673,7 +673,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / vehiclerental / gen6 / complex</t>
+          <t>gpt_4o / cot / videoclub / gen2 / edge</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -683,7 +683,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / restaurant / gen26</t>
+          <t>gpt_5_2 / simple / vehiclerental / gen12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -693,7 +693,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / videoclub / gen6</t>
+          <t>gpt_5_2 / simple / videoclub / gen27</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -703,7 +703,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / restaurant / gen4 / complex</t>
+          <t>gpt_4o / cot / myexpenses / gen1 / edge</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -713,7 +713,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / bank / gen13</t>
+          <t>gpt_4o / simple / bank / gen11</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -723,7 +723,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / myexpenses / gen5 / invalid</t>
+          <t>gpt_5_2 / cot / myexpenses / gen6 / boundary</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -733,7 +733,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / statemachine / gen4</t>
+          <t>gpt_4o / simple / statemachine / gen10</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -743,7 +743,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / videoclub / gen5 / boundary</t>
+          <t>gpt_5_2 / cot / videoclub / gen4 / edge</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -753,7 +753,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / football / gen1 / boundary</t>
+          <t>gpt_5_2 / cot / football / gen3 / edge</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -763,7 +763,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / pickupnet / gen4 / boundary</t>
+          <t>gpt_5_2 / cot / statemachine / gen5 / baseline</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -773,7 +773,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / restaurant / gen20</t>
+          <t>gpt_5_2 / simple / statemachine / gen14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -783,7 +783,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / videoclub / gen16</t>
+          <t>gpt_5_2 / simple / videoclub / gen30</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -793,7 +793,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / addressbook / gen10</t>
+          <t>gpt_5_2 / simple / addressbook / gen7</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -803,7 +803,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / hotelmanagement / gen1 / edge</t>
+          <t>gpt_4o / cot / football / gen3 / invalid</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -813,7 +813,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / restaurant / gen6 / boundary</t>
+          <t>gpt_4o / cot / myexpenses / gen6 / edge</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -823,7 +823,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / vehiclerental / gen27</t>
+          <t>gpt_4o / simple / vehiclerental / gen20</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -843,7 +843,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / statemachine / gen3</t>
+          <t>gpt_4o / simple / restaurant / gen10</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -930,7 +930,7 @@
             <t xml:space="preserve">0. </t>
           </r>
           <r>
-            <t>Review the following prompts to understand the criteria used during realism evaluation.</t>
+            <t>Review the judge prompts to understand the criteria used during realism evaluation.</t>
           </r>
         </is>
       </c>
@@ -939,7 +939,7 @@
       <c r="A3" s="2" t="inlineStr">
         <is>
           <r>
-            <t>System Judge: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=system-judge-prompt</t>
+            <t>Judge System Prompt: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=system-judge-prompt</t>
           </r>
         </is>
       </c>
@@ -948,7 +948,7 @@
       <c r="A4" s="2" t="inlineStr">
         <is>
           <r>
-            <t>User Judge: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=user-judge-prompt</t>
+            <t>Judge User Prompt: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=user-judge-prompt</t>
           </r>
         </is>
       </c>
@@ -1077,7 +1077,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / videoclub / gen2 / baseline</t>
+          <t>gpt_5_2 / cot / videoclub / gen3 / complex</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -1087,7 +1087,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / videoclub / gen2 / complex</t>
+          <t>gpt_4o / cot / videoclub / gen2 / baseline</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -1097,7 +1097,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / bank / gen5 / boundary</t>
+          <t>gpt_4o / cot / bank / gen4 / baseline</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -1107,7 +1107,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / statemachine / gen20</t>
+          <t>gpt_4o / simple / statemachine / gen12</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -1117,7 +1117,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / myexpenses / gen4 / baseline</t>
+          <t>gpt_5_2 / cot / pickupnet / gen6 / baseline</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -1127,7 +1127,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / videoclub / gen2 / baseline</t>
+          <t>gpt_4o / cot / videoclub / gen1 / invalid</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -1137,7 +1137,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / addressbook / gen17</t>
+          <t>gpt_4o / simple / addressbook / gen24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -1147,7 +1147,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / addressbook / gen20</t>
+          <t>gpt_5_2 / simple / addressbook / gen16</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -1157,7 +1157,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / addressbook / gen30</t>
+          <t>gpt_5_2 / simple / addressbook / gen25</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -1167,7 +1167,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / restaurant / gen10</t>
+          <t>gpt_5_2 / simple / vehiclerental / gen2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -1177,7 +1177,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / football / gen21</t>
+          <t>gpt_4o / simple / hotelmanagement / gen19</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -1187,7 +1187,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / pickupnet / gen11</t>
+          <t>gpt_4o / simple / pickupnet / gen7</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -1197,7 +1197,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / addressbook / gen1 / boundary</t>
+          <t>gpt_5_2 / cot / addressbook / gen1 / edge</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -1217,7 +1217,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / football / gen2 / complex</t>
+          <t>gpt_5_2 / cot / football / gen1 / baseline</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -1227,7 +1227,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / vehiclerental / gen5 / boundary</t>
+          <t>gpt_5_2 / cot / restaurant / gen6 / invalid</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -1237,7 +1237,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / pickupnet / gen2</t>
+          <t>gpt_5_2 / simple / restaurant / gen8</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / hotelmanagement / gen3 / baseline</t>
+          <t>gpt_4o / cot / football / gen4 / complex</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -1257,7 +1257,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / addressbook / gen11</t>
+          <t>gpt_5_2 / simple / addressbook / gen14</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -1267,7 +1267,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / hotelmanagement / gen5 / complex</t>
+          <t>gpt_5_2 / cot / hotelmanagement / gen1 / invalid</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1277,7 +1277,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / restaurant / gen1</t>
+          <t>gpt_4o / simple / restaurant / gen3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1287,7 +1287,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / statemachine / gen1 / boundary</t>
+          <t>gpt_4o / cot / statemachine / gen2 / complex</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1297,7 +1297,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / pickupnet / gen23</t>
+          <t>gpt_5_2 / simple / restaurant / gen22</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1307,7 +1307,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / hotelmanagement / gen13</t>
+          <t>gpt_4o / simple / pickupnet / gen13</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1394,7 +1394,7 @@
             <t xml:space="preserve">0. </t>
           </r>
           <r>
-            <t>Review the following prompts to understand the criteria used during realism evaluation.</t>
+            <t>Review the judge prompts to understand the criteria used during realism evaluation.</t>
           </r>
         </is>
       </c>
@@ -1403,7 +1403,7 @@
       <c r="A3" s="2" t="inlineStr">
         <is>
           <r>
-            <t>System Judge: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=system-judge-prompt</t>
+            <t>Judge System Prompt: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=system-judge-prompt</t>
           </r>
         </is>
       </c>
@@ -1412,7 +1412,7 @@
       <c r="A4" s="2" t="inlineStr">
         <is>
           <r>
-            <t>User Judge: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=user-judge-prompt</t>
+            <t>Judge User Prompt: https://a-coman.github.io/llm-viewer/gpt_4o/bank/gen1/?view=user-judge-prompt</t>
           </r>
         </is>
       </c>
@@ -1541,7 +1541,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / pickupnet / gen4 / invalid</t>
+          <t>gpt_4o / cot / hotelmanagement / gen1 / invalid</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -1551,7 +1551,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / restaurant / gen6 / edge</t>
+          <t>gpt_5_2 / cot / restaurant / gen1 / edge</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -1561,7 +1561,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / vehiclerental / gen19</t>
+          <t>gpt_4o / simple / vehiclerental / gen17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -1571,7 +1571,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / football / gen8</t>
+          <t>gpt_4o / simple / football / gen18</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -1581,7 +1581,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / statemachine / gen2 / boundary</t>
+          <t>gpt_4o / cot / statemachine / gen6 / edge</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -1591,7 +1591,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / statemachine / gen15</t>
+          <t>gpt_5_2 / simple / videoclub / gen6</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -1611,7 +1611,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / statemachine / gen29</t>
+          <t>gpt_4o / simple / vehiclerental / gen13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -1621,7 +1621,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / videoclub / gen2 / edge</t>
+          <t>gpt_4o / cot / videoclub / gen2 / invalid</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -1631,7 +1631,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / vehiclerental / gen8</t>
+          <t>gpt_4o / simple / restaurant / gen27</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -1641,7 +1641,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / bank / gen20</t>
+          <t>gpt_5_2 / simple / myexpenses / gen4</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -1651,7 +1651,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / vehiclerental / gen21</t>
+          <t>gpt_5_2 / simple / videoclub / gen7</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -1661,7 +1661,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / myexpenses / gen4 / edge</t>
+          <t>gpt_5_2 / cot / restaurant / gen2 / boundary</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -1671,7 +1671,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / restaurant / gen2 / baseline</t>
+          <t>gpt_5_2 / cot / vehiclerental / gen1 / baseline</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -1681,7 +1681,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / hotelmanagement / gen1 / baseline</t>
+          <t>gpt_4o / cot / myexpenses / gen3 / complex</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -1691,7 +1691,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / restaurant / gen3 / baseline</t>
+          <t>gpt_5_2 / cot / pickupnet / gen3 / invalid</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -1701,7 +1701,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / statemachine / gen3 / edge</t>
+          <t>gpt_4o / cot / vehiclerental / gen1 / complex</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -1711,7 +1711,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / restaurant / gen8</t>
+          <t>gpt_4o / simple / statemachine / gen3</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -1721,7 +1721,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / simple / bank / gen17</t>
+          <t>gpt_4o / simple / football / gen6</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -1731,7 +1731,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / statemachine / gen4 / edge</t>
+          <t>gpt_4o / cot / videoclub / gen1 / baseline</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1741,7 +1741,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>gpt_4o / cot / statemachine / gen4 / baseline</t>
+          <t>gpt_4o / cot / vehiclerental / gen2 / complex</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1751,7 +1751,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / hotelmanagement / gen6 / baseline</t>
+          <t>gpt_5_2 / cot / hotelmanagement / gen3 / boundary</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1761,7 +1761,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / cot / pickupnet / gen4 / complex</t>
+          <t>gpt_5_2 / cot / statemachine / gen6 / boundary</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1771,7 +1771,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>gpt_5_2 / simple / restaurant / gen11</t>
+          <t>gpt_5_2 / simple / vehiclerental / gen5</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>

</xml_diff>

<commit_message>
Add judge_random_eval py script and update card to be automatically expanded
</commit_message>
<xml_diff>
--- a/src/scripts/random_eval_1.xlsx
+++ b/src/scripts/random_eval_1.xlsx
@@ -435,13 +435,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="64" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -602,6 +603,7 @@
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -622,6 +624,11 @@
       <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Manuel</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Gemini 3.1 Pro</t>
         </is>
       </c>
     </row>
@@ -634,6 +641,11 @@
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>U: The relationship 'relationship23' defines a 'SUBDIVISION' connection between a Company ('company12') and a Person ('person20'). In the real world, a person cannot be a subdivision of a company; a subdivision refers to a department or subsidiary business unit. An 'EMPLOYEE' or 'BOSS' relationship would be appropriate instead.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -644,6 +656,11 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>U: The 'FoodItem' object 'foodItem20' (described as 'Organic Eggs') is associated with the 'Allergen' object 'allergen20' of type 'Lactose'. Biologically, eggs are not dairy products and do not contain lactose.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -654,6 +671,11 @@
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>U: The object 'room13_101' has a 'pricePerNight' of 0.0, which is unrealistic for a hotel room's catalog rate. Furthermore, 'roomReservation13_2' is linked to this free room along with 200.0 in extras, yet it generates two separate bills ('bill27' at 500.0 and 'bill28' at 400.0) totaling 900.0, which is mathematically contradictory. Finally, associating two bills to 'roomReservation13_2' directly violates the strictly 1-to-1 multiplicity of the 'BillRoomReservation' association.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -664,6 +686,11 @@
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>U: The model contains a logical contradiction within the given domain. The expense 'expensePerDiemOnlyDakar' is assigned an amount of 120.00 but has no associated bills. This directly violates the domain constraint 'expenseSumOfBills', which requires the expense amount to equal the sum of its bills' amounts (which would be 0.0 here).</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -674,6 +701,11 @@
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>U: The relationship 'CarlosToAikoSubdivision' assigns the type '#SUBDIVISION' between two 'Person' objects ('DrCarlosMendes' and 'ProfAikoTanaka'). In reality, a person cannot be a subdivision of another person. Additionally, the relationship 'SpaceToAikoCoworker' designates a 'Company' ('InternationalSpaceResearchAgency') and a 'Person' as coworkers, which is logically impossible as organizations and human beings do not share a coworker dynamic.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -684,6 +716,11 @@
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>R: The object model is highly consistent. The names of the individuals culturally align with the countries of their respective banks (Greek names for the National Bank of Greece, and an English/NZ name for Kiwibank). The IBAN country codes match the bank locations, the balances are positive, the owners are adults, and co-ownership and authorized user relationships are logically structured.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -694,6 +731,11 @@
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>R: The object model is semantically consistent and highly plausible. The attribute values (such as distances, gas tank capacity, and pricing) are common-sense and appropriate for a vehicle rental system. The scenario logically models a standard rental use case, including a realistic one-way 6-day truck rental from Connecticut to Colorado, which realistically returns the vehicle to its home office.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -704,6 +746,11 @@
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>R: The object model uses valid strings, logical dates (2023-12-07), and plausible integer values for available copies and identifiers. The relationships correctly and naturally map clients to their rentals, rentals to movies, and actors to their respective movies. Having a rental assigned to a suspended client is realistic in a snapshot, as they are likely suspended for not returning the rented cassette.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -714,6 +761,11 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>R: The object model is semantically consistent and highly detailed. Attributes like addresses, states, and vehicle types align perfectly (e.g., a Florida office managing a Florida-registered truck). The relationships describe logical real-world rental scenarios, such as a 4-day one-way truck rental from Miami to Denver, and a local 2-day flat-rate trailer rental (with a $0.00 rate per mile, which is accurate for trailers since they lack odometers). Values for truck gas tank capacity (26.5), mileage/MPG (17), and daily rates are standard and plausible.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -724,6 +776,11 @@
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>R: The object model represents a plausible real-world scenario. The rentals involve realistic combinations of cassettes (e.g., sequentially borrowing multiple episodes of the "Northern Lights" series). It is logically sound that a client like 'cz3' who has an outstanding rental with multiple cassettes might have an 'isSuspended' status set to true due to unreturned items.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -734,6 +791,11 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>R: The assigned attributes have plausible real-world values. The dates of the bills correctly fall within the start and end dates of the overarching expense. The sum of the individual bill amounts (4000 + 3000 + 2000) correctly totals the expense amount (9000), and the currencies, categories, and payment methods represent sensible financial data.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -744,6 +806,11 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>R: The object model is logically consistent and adheres to the domain model's constraints. The attributes reflect plausible real-world values (e.g., table capacities match the number of people in the reservations, employee ages and roles are perfectly valid), and all necessary multiplicity constraints are satisfied for a snapshot in time. Using a placeholder phone number and a 0.0 prep time for a "zero-prep demo" item are both common, valid scenarios in a real system.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -754,6 +821,11 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>R: The object model defines two entirely plausible state machines: a clinic appointment flow and a continuous integration (CI) pipeline. The states are logically named and follow standard real-world lifecycles. The transitions connect appropriate states, and the time values assigned to events are logically consistent (e.g., 1440 minutes/1 day from scheduled to check-in, 15 minutes in the waiting room, standard CI build/test/deploy steps). All domain constraints are satisfied.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -764,6 +836,11 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>R: The object model provides a logically consistent and temporally valid set of business entities. Attributes like gas tank capacity, odometer readings, and rental rates are well within plausible real-world boundaries. The rental agreements follow a clear chronological sequence without overlapping a single vehicle's usage across physically distant rental periods.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -774,6 +851,11 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>U: The stay dates for the reservation are from December 20th to December 25th, but the booked room extra 'extra17' is a "New Year Celebration Package". It is logically inconsistent to book a New Year's package for a stay that concludes on Christmas Day, well before the New Year.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -784,6 +866,11 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>R: The object model is logically consistent with the domain model and represents a plausible real-world scenario for a video club. Client IDs, rental dates, and episode numbers are valid. Multiplicities and constraints are fully respected. Attributes like available copies and overlapping actors in different episodes correctly mirror real-world behaviors. The presence of a suspended client with a past rental is also a valid business scenario (e.g., suspended due to unreturned items).</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -794,6 +881,11 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>U: The relationships between objects are logically nonsensical. A person ('SantiagoReyes') cannot have a company ('GlobalArtMovement') as a 'SUBDIVISION', nor can an educational institution or company ('ArtHavenAcademy') act as an 'EMPLOYEE' to a person. Furthermore, companies ('GlobalArtMovement' and 'ArtHavenAcademy') are related as 'COWORKER's, which is a term reserved for individuals.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -804,6 +896,11 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>R: The object model accurately represents a real-world clinical MRI workflow. The states logically progress through the procedural phases (e.g., registration, screening, preparation, sequencing of scans, contrast injection, and disinfection). Alternate paths handling real-life exceptions, such as metal implant issues, motion artifacts, or allergic reactions, are logically routed. The time events mapped to each transition represent highly plausible durations (in minutes) for these medical tasks. All UML constraints are satisfied.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -814,6 +911,11 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>U: The state 'st_carn_concentracao' has five different outgoing transitions (towards 'setorA', 'setorB', 'setorC', and 'apuracao'), and all of them are triggered by a `TimeEvent` with the exact same time (`time := 1`). In a state machine, this creates unresolvable non-determinism, as the system would attempt to transition to five mutually exclusive states at the exact same moment. Additionally, the state 'st_carn_vipLounge' is completely isolated with no incoming or outgoing transitions.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -824,18 +926,23 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>U: The objects 'K55' and 'K56' of class 'Cook' are instantiated as two distinct objects but share the exact same name ('Pavel Novák'), date of birth ('1993-03-03'), and personal phone number ('+420 2 700 2001'). In reality, this implies the exact same physical human being has been duplicated into two separate entities within the model, which violates object identity principles.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
@@ -871,13 +978,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="64" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1038,6 +1146,7 @@
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1058,6 +1167,11 @@
       <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Dominik</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Gemini 3.1 Pro</t>
         </is>
       </c>
     </row>
@@ -1070,6 +1184,11 @@
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>R: The client, actor, and cassette properties are completely plausible and consistent with real-world entities. The scenario where a suspended client ('vb') retains a rental ('vxR1') of series episodes with 0 available copies perfectly reflects common real-world logic for a video club snapshot.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1080,6 +1199,11 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>U: The address texts ('Spaceport Alpha', 'Xandar') are fictional, interstellar locations, yet they are mapped to standard Earth geolocation coordinates (Mumbai and Borneo). Additionally, a single localized 'Station' (station26) is managing drivers and shipments spanning thousands of kilometers, which contradicts the real-world logistical function of a delivery station.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1090,6 +1214,11 @@
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>U: The shipment statuses contradict their real-world logistical relationships. Object 'shipment41' has the status 'NEW' despite already being assigned to 'driver38' (it should be at least 'ASSIGNED'). Conversely, 'shipment42' has the status 'DELIVERED', but lacks any associated driver in the 'DriverShipment' relationship to have actually performed the delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1100,6 +1229,11 @@
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>U: The account 'a103' has a balance of exactly 2147483647, which represents the maximum value of a 32-bit signed integer. While syntactically valid, this is a recognizable software testing artifact rather than a naturally occurring, plausible real-world bank account balance.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1110,6 +1244,11 @@
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>U: The relationship 'relationship25' designates 'person22' (a Person) as a 'SUBDIVISION' of 'company13' (a Company). In the real world, a subdivision is a structural branch or department (typified as another Company or organization), whereas an individual should use the 'EMPLOYEE' or 'BOSS' relationship types.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1120,6 +1259,11 @@
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>R: The assigned attribute values are plausible for real-world individuals and banking entities. Ages are over 18, the balance is positive, and the relationships appropriately reflect real-world scenarios where bank accounts can be jointly owned and used by authorized non-owners.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1130,6 +1274,11 @@
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>U: The booking 'booking16' is marked as unconfirmed and canceled, yet its associated room reservation 'rr22' includes charges for on-site physical consumption like 'Late room service' and 'Express cleaning'. It is a logical contradiction to incur on-site service bills for a stay that was never confirmed or took place (additionally, the dates are in the future).</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1140,6 +1289,11 @@
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>U: The object model contains severe logical contradictions and category errors in its relationships. For example, `P_Archivist_1` is simultaneously modeled as a BOSS and an EMPLOYEE of `P_Haakon_1`. Furthermore, `P_Archivist_1` (a Person) is related to `C_MicroEtats_1` and `C_Paperless_1` (Companies) via a SUBDIVISION relationship, which makes no sense in the real world as a person cannot be a structural subdivision of a company. The notes in the objects even explicitly admit it is a contradictory test dataset.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1150,6 +1304,11 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>U: The physical logistics are implausible. The objects 'table9' and 'table10' each have a capacity of 150, which is absurdly large for single physical restaurant tables. Additionally, assigning only 2 waiters ('waiter5', 'waiter6') to serve a 300-person banquet defies real-world restaurant staffing logic, and 1 bus driver ('busdriver3') cannot transport 300 people simultaneously.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1160,6 +1319,11 @@
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>R: The amounts and categories align well with standard R&amp;D expenses. The total expense amount correctly matches the sum of the individual bills (1,800,000 KRW), and the dates of the bills all logically fall within the expense's start and end dates. The currency matches a real-world fiat currency with appropriate values.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1170,6 +1334,11 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>U: The object 'account21' has a Norwegian IBAN ('NO9386011117948') but is associated with 'bank14' (Banco Galicia), which is an Argentine bank. In the real world, an account's IBAN country code must match the country of the issuing bank.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1180,6 +1349,11 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>R: The object model represents a plausible real-world hotel booking scenario. The dates for the booking and check-in/out match logically, room attributes and pricing ($120/night, 2 beds) are typical, and extras like 'Gym Access' or 'Welcome Drink' with their respective prices make perfect sense within a hotel context. The billed amount is also within a realistic range for the stay length.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1190,6 +1364,11 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>R: The object model represents a highly plausible scenario. The instances properly reflect real-world values, such as accurate Oregon area codes (503) and zip codes for the cities listed. The chronological alignment of maintenance, expiration, and rental dates is completely logical, and combinations of durations, daily rates, and deposits are mathematically sound and standard for the rental industry. No physical or logical domain constraints are violated.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1200,6 +1379,11 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>R: The object model represents a highly plausible finite state machine for a robot. The states (standby, operational, errorMode, etc.) and transitions logically follow real-world equipment lifecycles. All domain constraints, multiplicities, positive time values, and lowercase naming conventions are strictly and appropriately followed.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1210,6 +1394,11 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>U: The object model is syntactically incomplete and violates the domain model's cardinality constraints. The composition `StationContainsCustomer` dictates that every `Customer` must be associated with exactly one `Station` (multiplicity `Station [1]`), but the object `customer17` is created without ever being linked to a Station.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1220,6 +1409,11 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>R: The object model is syntactically correct and semantically logical. The geographic coordinates accurately map to the Delhi-NCR region, the addresses match real-world locations, and the assignment of drivers corresponds correctly to the shipment statuses (i.e., 'NEW' shipments lack a driver, while other statuses have one). All constraints, including unique IDs and distinct pickup/delivery addresses, are satisfied.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1230,6 +1424,11 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>U: Player 'player51' failed to attend 'trainingSession38' via the 'trainingFail15' record. However, 'player51' belongs to 'teamAS', while 'trainingSession38' is a training session for a different team ('teamAR'). A player cannot be marked as failing to attend a training session for a team they do not play for.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1240,6 +1439,11 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>U: The transition 'transition22' is named 'startQualityCheck', but its source is the 'qualityCheck' state and its target is the 'rawMaterials' state. Logically, a transition named 'startQualityCheck' should target the 'qualityCheck' state, not depart from it.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1250,6 +1454,11 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>R: The object model demonstrates strong semantic consistency with real-world rental business logic. For instance, trailers are logically assigned a $0.00 per-mile rate because they lack odometers, while trucks have appropriate per-mile charges, realistic MPG (mileage), and gas tank capacities. State identifiers, license plates, and branch locations correctly correspond to one another, and all multiplicity and domain constraints are fully satisfied.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1260,18 +1469,23 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>R: The object model represents a valid, plausible state of a delivery network (a station containing several customers and a driver). The attribute values for names, distinct IDs, and Twitter handles (properly formatted with '@') are completely realistic, and the relationships respect the domain model's logic.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
@@ -1307,13 +1521,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="64" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1474,6 +1689,7 @@
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1494,6 +1710,11 @@
       <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Lola</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Gemini 3.1 Pro</t>
         </is>
       </c>
     </row>
@@ -1506,6 +1727,11 @@
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>U: The banquet reservation 'banq12' has 120 people attending but is assigned to be served by only a single waiter ('w34'). It is physically impossible for one person to serve a banquet of this size, especially set against the fact that a much smaller reservation of 8 people ('res20') correctly utilizes two waiters.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1516,6 +1742,11 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>U: The expense 'expSepFilmProduction' sums up bills of different currencies (Ugandan Shilling and Sri Lankan Rupee) by directly adding their raw numerical values without any exchange rate conversion, which is financially nonsensical. Additionally, the amounts are drastically unrealistic for the chosen currencies (e.g., 450 UGX for a camera rig rental is approximately $0.12 USD).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1526,6 +1757,11 @@
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>U: The object model violates the domain's explicit OCL constraint `TeamsFromDifferentClubs`. Match 'M9' is played between the local team 'T15' and the visitor team 'T16', but both of these teams belong to the exact same club ('C14'), which contradicts the constraints.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1536,6 +1772,11 @@
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>U: The state machines 'smGreenStart', 'smYellowStart', and 'smOpenStart' do not contain any states themselves, yet they define states belonging to other state machines ('smTraffic' and 'smDoor') as their starting states. In state machine semantics, a start state must be contained within the state machine it initiates.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1546,6 +1787,11 @@
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>R: The object model is entirely plausible and logically consistent for a football tracking system. Attribute values such as 90 minutes for match duration, ages in the mid-20s for players, 0-0 match scores aligning correctly with the lack of goal events, and the realistic descriptive fields (e.g., 'Overtime at work') consistently follow real-world football and team management logic.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1556,6 +1802,11 @@
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>U: The match report states a final score of 3-3 (6 total goals), but there are only 3 match events of type GOAL created and linked to the match, creating a mathematical contradiction between the match score and the recorded goal events.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1566,6 +1817,11 @@
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>U: The object 'D16' of class 'FreeRoomTypesDTO' indicates there are 250 free "Presidential family suite" rooms with 12 beds each. A "Presidential suite" is by definition the most exclusive and limited accommodation in a hotel, typically restricted to one or a very small handful per property. Having 250 of them available is physically and economically nonsensical for a real-world hotel scenario.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1576,6 +1832,11 @@
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>U: The total amount for the 'artExhibitionLaunchExpense' (33400.00) is calculated by directly summing the raw face values of its associated bills (12000 + 8500 + 9000 + 3900), despite each bill being in an entirely different real-world currency (GBP, EUR, USD, JPY). Summing different monetary currencies 1:1 without exchange rate conversions is an economic and logical fallacy.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1586,6 +1847,11 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>U: The shipment 'shp_310004' has its status set to 'ASSIGNED', but it is not linked to any Driver object via the 'DriverShipment' association. In this domain context, transitioning from 'NEW' to 'ASSIGNED' logically requires the assignment of a delivery agent (Driver).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1596,6 +1862,11 @@
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>U: It is highly implausible in a real-world scenario that a single 18-year-old ('p105', Laura Gomez) would be granted 'Use' access to every bank account in the system ('accCH10' to 'accCH13'), which belong to several completely unrelated adults. Additionally, the assigned BIC code for 'bankCO1' ('BBNORCOBXXXX') is 12 characters long, whereas valid standard SWIFT/BIC codes are strictly 8 or 11 characters.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1606,6 +1877,11 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>R: The object model portrays a highly consistent and plausible restaurant scenario. All attributes accurately reflect real-world values (e.g., sensible prep times, matching food measurements like 'Ounce' for fluids and 'Sheet' for wrappers, logical ages, and sequential reservation/order times). Furthermore, the objects fully comply with the required multiplicities, capacities, and constraints (such as the sum of owner shares equaling 100). The instantiated objects without associations (DietaryRequirement, ReportedAllergy) simply stem from a lack of associations in the domain model, but their values remain logical.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1616,6 +1892,11 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>R: The data provided aligns perfectly with real-world banking scenarios. All people are adults with plausible ages, account balances are non-negative, and IBAN prefixes ('DE' and 'ZA') logically correspond to the banks' host countries (Germany and South Africa). The distinction between 'Ownership' and 'Use' realisticly models joint accounts and authorized user access (like a power of attorney).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1626,6 +1907,11 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>U: The relationship objects 'relGreenfieldCoworkerStonebridge' and 'relStonebridgeCoworkerGreenfield' assign a 'COWORKER' relationship type between 'greenfieldPrint' and 'stonebridgePublishing'. Both of these objects are instances of 'Company'. In the real world, individuals (Persons) can be coworkers, but corporate entities cannot.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1636,6 +1922,11 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>R: The object model represents a plausible hotel booking scenario. The attribute values for prices, dates, room capacities, and customer names are realistic. A canceled, unconfirmed booking can still have an associated bill (e.g., representing a deposit or cancellation fee) and specific rooms tied to the reservation history.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1646,6 +1937,11 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>R: The object model represents a plausible football scenario. Player ages (23 and 27) and attributes are standard. The match duration is exactly 90 minutes. The match scores (2-1) logically align with the exact number of 'GOAL' events recorded in the match (3 goals), and the goal times (20, 55, and 75) all mathematically fall within the match duration constraints.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1656,6 +1952,11 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>R: The object model represents a plausible real-world football scenario. The teams belong to different clubs, player ages and positions are realistic, match details including duration and player ratings (7 and 9) are sensible, and exactly six 'GOAL' events are recorded, perfectly matching the final match report score of 3-3.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1666,6 +1967,11 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>R: The object model represents a standard, plausible scenario for a video club. Creating clients, rentals across valid dates, movies, and series with positive available copies and episode numbers, and associating them with actors follows real-world logic perfectly. Everything aligns with the constraints and logical business rules of a rental store.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1676,6 +1982,11 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>R: The object model portrays a completely consistent real-world scenario of submitting an expense report for a fully refunded purchase. The bill date (2023-12-10) falls logically within the expense period (December 2023), the currency represents a valid real-world currency (Canadian Dollar/CAD), the expense amount accurately equals the sum of the bills (0), and the comment logically explains the 0.00 amounts.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1686,6 +1997,11 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>R: The object model represents a plausible scenario with valid real-world attributes (human names, reasonable dates, realistic titles, and correct quantities). The relationships correctly assign un-suspended clients to rentals, and the multiplicities accurately reflect a functioning video club system.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1696,18 +2012,23 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>R: The assigned attribute values and relationships represent a plausible real-world vehicle rental scenario. Prices, deposits, daily rates (~$70/day), vehicle attributes (like ~33 gallon gas tanks and ~20 MPG mileage), and standard round-trip rental office associations are all logically consistent and within expected realistic bounds.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>

</xml_diff>